<commit_message>
did stuff for heat ransfer
</commit_message>
<xml_diff>
--- a/two_boiling.xlsx
+++ b/two_boiling.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I227"/>
+  <dimension ref="A1:I236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.71428571428572" customWidth="1" min="1" max="1"/>
@@ -2023,1314 +2023,1257 @@
         </is>
       </c>
     </row>
-    <row r="113" ht="17" customHeight="1">
-      <c r="A113" s="4" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="18" t="inlineStr">
+        <is>
+          <t>Heating surface</t>
+        </is>
+      </c>
+      <c r="B112" s="22" t="n">
+        <v>22500</v>
+      </c>
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t>ft²</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="18" t="inlineStr">
+        <is>
+          <t>dT (calandria - masse)</t>
+        </is>
+      </c>
+      <c r="B113" s="23" t="n">
+        <v>46.73119721756075</v>
+      </c>
+      <c r="C113" s="20" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="18" t="inlineStr">
+        <is>
+          <t>Overall U (back-calc)</t>
+        </is>
+      </c>
+      <c r="B114" s="23" t="n">
+        <v>71.4844431192349</v>
+      </c>
+      <c r="C114" s="20" t="inlineStr">
+        <is>
+          <t>BTU/hr·ft²·°F</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="17" customHeight="1">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>A CENTRIFUGALS  [A Centrifugals]</t>
         </is>
       </c>
-      <c r="B113" s="5" t="n"/>
-      <c r="C113" s="5" t="n"/>
-      <c r="D113" s="5" t="n"/>
-      <c r="E113" s="5" t="n"/>
-      <c r="F113" s="5" t="n"/>
-      <c r="G113" s="5" t="n"/>
-      <c r="H113" s="5" t="n"/>
-      <c r="I113" s="5" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="6" t="inlineStr">
+      <c r="B116" s="5" t="n"/>
+      <c r="C116" s="5" t="n"/>
+      <c r="D116" s="5" t="n"/>
+      <c r="E116" s="5" t="n"/>
+      <c r="F116" s="5" t="n"/>
+      <c r="G116" s="5" t="n"/>
+      <c r="H116" s="5" t="n"/>
+      <c r="I116" s="5" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B114" s="6" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>Dir</t>
         </is>
       </c>
-      <c r="C114" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>Flow (lb/hr)</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>Solids (lb/hr)</t>
         </is>
       </c>
-      <c r="E114" s="6" t="inlineStr">
+      <c r="E117" s="6" t="inlineStr">
         <is>
           <t>Pol (lb/hr)</t>
         </is>
       </c>
-      <c r="F114" s="6" t="inlineStr">
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>Water (lb/hr)</t>
         </is>
       </c>
-      <c r="G114" s="6" t="inlineStr">
+      <c r="G117" s="6" t="inlineStr">
         <is>
           <t>Brix %</t>
         </is>
       </c>
-      <c r="H114" s="6" t="inlineStr">
+      <c r="H117" s="6" t="inlineStr">
         <is>
           <t>Purity %</t>
         </is>
       </c>
-      <c r="I114" s="6" t="inlineStr">
+      <c r="I117" s="6" t="inlineStr">
         <is>
           <t>ft³/hr</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="8" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
         <is>
           <t>Massecuite</t>
         </is>
       </c>
-      <c r="B115" s="8" t="inlineStr">
+      <c r="B118" s="8" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C115" s="9" t="n">
+      <c r="C118" s="9" t="n">
         <v>179587.0508851917</v>
       </c>
-      <c r="D115" s="9" t="n">
+      <c r="D118" s="9" t="n">
         <v>165220.0868143764</v>
       </c>
-      <c r="E115" s="9" t="n">
+      <c r="E118" s="9" t="n">
         <v>122701.3198984672</v>
       </c>
-      <c r="F115" s="9" t="n">
+      <c r="F118" s="9" t="n">
         <v>14366.96407081533</v>
       </c>
-      <c r="G115" s="10" t="n">
+      <c r="G118" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="H115" s="10" t="n">
+      <c r="H118" s="10" t="n">
         <v>74.26537672524117</v>
       </c>
-      <c r="I115" s="9" t="n">
+      <c r="I118" s="9" t="n">
         <v>1926.728261085383</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="12" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="12" t="inlineStr">
         <is>
           <t>Wash Water</t>
         </is>
       </c>
-      <c r="B116" s="12" t="inlineStr">
+      <c r="B119" s="12" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C116" s="13" t="n">
+      <c r="C119" s="13" t="n">
         <v>7334.960534310288</v>
       </c>
-      <c r="D116" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E116" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F116" s="13" t="n">
+      <c r="D119" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" s="13" t="n">
         <v>7334.960534310288</v>
       </c>
-      <c r="G116" s="12" t="inlineStr"/>
-      <c r="H116" s="12" t="inlineStr"/>
-      <c r="I116" s="12" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="inlineStr">
+      <c r="G119" s="12" t="inlineStr"/>
+      <c r="H119" s="12" t="inlineStr"/>
+      <c r="I119" s="12" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t>Sugar Out</t>
         </is>
       </c>
-      <c r="B117" s="8" t="inlineStr">
+      <c r="B120" s="8" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C117" s="9" t="n">
+      <c r="C120" s="9" t="n">
         <v>67480.43757279526</v>
       </c>
-      <c r="D117" s="9" t="n">
+      <c r="D120" s="9" t="n">
         <v>67277.99626007688</v>
       </c>
-      <c r="E117" s="9" t="n">
+      <c r="E120" s="9" t="n">
         <v>66874.32828251641</v>
       </c>
-      <c r="F117" s="9" t="n">
+      <c r="F120" s="9" t="n">
         <v>202.4413127183798</v>
       </c>
-      <c r="G117" s="10" t="n">
+      <c r="G120" s="10" t="n">
         <v>99.7</v>
       </c>
-      <c r="H117" s="10" t="n">
+      <c r="H120" s="10" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="I117" s="9" t="n">
+      <c r="I120" s="9" t="n">
         <v>697.9842931297231</v>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="12" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="12" t="inlineStr">
         <is>
           <t>Molasses Out</t>
         </is>
       </c>
-      <c r="B118" s="12" t="inlineStr">
+      <c r="B121" s="12" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C118" s="13" t="n">
+      <c r="C121" s="13" t="n">
         <v>119441.5738467068</v>
       </c>
-      <c r="D118" s="13" t="n">
+      <c r="D121" s="13" t="n">
         <v>97942.09055429955</v>
       </c>
-      <c r="E118" s="13" t="n">
+      <c r="E121" s="13" t="n">
         <v>55826.99161595074</v>
       </c>
-      <c r="F118" s="13" t="n">
+      <c r="F121" s="13" t="n">
         <v>21499.48329240721</v>
       </c>
-      <c r="G118" s="14" t="n">
+      <c r="G121" s="14" t="n">
         <v>82</v>
       </c>
-      <c r="H118" s="14" t="n">
+      <c r="H121" s="14" t="n">
         <v>57</v>
       </c>
-      <c r="I118" s="13" t="n">
+      <c r="I121" s="13" t="n">
         <v>1343.558979194719</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="17" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="17" t="inlineStr">
         <is>
           <t>Total In</t>
         </is>
       </c>
-      <c r="B119" s="17" t="inlineStr"/>
-      <c r="C119" s="16" t="n">
+      <c r="B122" s="17" t="inlineStr"/>
+      <c r="C122" s="16" t="n">
         <v>186922.011419502</v>
       </c>
-      <c r="D119" s="16" t="n">
+      <c r="D122" s="16" t="n">
         <v>165220.0868143764</v>
       </c>
-      <c r="E119" s="16" t="n">
+      <c r="E122" s="16" t="n">
         <v>122701.3198984672</v>
       </c>
-      <c r="F119" s="16" t="n">
+      <c r="F122" s="16" t="n">
         <v>21701.92460512562</v>
       </c>
-      <c r="G119" s="17" t="inlineStr"/>
-      <c r="H119" s="17" t="inlineStr"/>
-      <c r="I119" s="17" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="17" t="inlineStr">
+      <c r="G122" s="17" t="inlineStr"/>
+      <c r="H122" s="17" t="inlineStr"/>
+      <c r="I122" s="17" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="inlineStr">
         <is>
           <t>Total Out</t>
         </is>
       </c>
-      <c r="B120" s="17" t="inlineStr"/>
-      <c r="C120" s="16" t="n">
+      <c r="B123" s="17" t="inlineStr"/>
+      <c r="C123" s="16" t="n">
         <v>186922.011419502</v>
       </c>
-      <c r="D120" s="16" t="n">
+      <c r="D123" s="16" t="n">
         <v>165220.0868143764</v>
       </c>
-      <c r="E120" s="16" t="n">
+      <c r="E123" s="16" t="n">
         <v>122701.3198984671</v>
       </c>
-      <c r="F120" s="16" t="n">
+      <c r="F123" s="16" t="n">
         <v>21701.92460512562</v>
       </c>
-      <c r="G120" s="17" t="inlineStr"/>
-      <c r="H120" s="17" t="inlineStr"/>
-      <c r="I120" s="17" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="17" t="inlineStr">
+      <c r="G123" s="17" t="inlineStr"/>
+      <c r="H123" s="17" t="inlineStr"/>
+      <c r="I123" s="17" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="inlineStr">
         <is>
           <t>Net (In - Out)</t>
         </is>
       </c>
-      <c r="B121" s="17" t="inlineStr"/>
-      <c r="C121" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D121" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E121" s="16" t="n">
+      <c r="B124" s="17" t="inlineStr"/>
+      <c r="C124" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" s="16" t="n">
         <v>1.455191522836685e-11</v>
       </c>
-      <c r="F121" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G121" s="17" t="inlineStr"/>
-      <c r="H121" s="17" t="inlineStr"/>
-      <c r="I121" s="17" t="inlineStr"/>
-    </row>
-    <row r="123" ht="17" customHeight="1">
-      <c r="A123" s="4" t="inlineStr">
+      <c r="F124" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" s="17" t="inlineStr"/>
+      <c r="H124" s="17" t="inlineStr"/>
+      <c r="I124" s="17" t="inlineStr"/>
+    </row>
+    <row r="126" ht="17" customHeight="1">
+      <c r="A126" s="4" t="inlineStr">
         <is>
           <t>A MOLASSES DILUTION  (target 70.0 Bx)</t>
         </is>
       </c>
-      <c r="B123" s="5" t="n"/>
-      <c r="C123" s="5" t="n"/>
-      <c r="D123" s="5" t="n"/>
-      <c r="E123" s="5" t="n"/>
-      <c r="F123" s="5" t="n"/>
-      <c r="G123" s="5" t="n"/>
-      <c r="H123" s="5" t="n"/>
-      <c r="I123" s="5" t="n"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="6" t="inlineStr">
+      <c r="B126" s="5" t="n"/>
+      <c r="C126" s="5" t="n"/>
+      <c r="D126" s="5" t="n"/>
+      <c r="E126" s="5" t="n"/>
+      <c r="F126" s="5" t="n"/>
+      <c r="G126" s="5" t="n"/>
+      <c r="H126" s="5" t="n"/>
+      <c r="I126" s="5" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B124" s="6" t="inlineStr">
+      <c r="B127" s="6" t="inlineStr">
         <is>
           <t>Dir</t>
         </is>
       </c>
-      <c r="C124" s="6" t="inlineStr">
+      <c r="C127" s="6" t="inlineStr">
         <is>
           <t>Flow (lb/hr)</t>
         </is>
       </c>
-      <c r="D124" s="6" t="inlineStr">
+      <c r="D127" s="6" t="inlineStr">
         <is>
           <t>Solids (lb/hr)</t>
         </is>
       </c>
-      <c r="E124" s="6" t="inlineStr">
+      <c r="E127" s="6" t="inlineStr">
         <is>
           <t>Pol (lb/hr)</t>
         </is>
       </c>
-      <c r="F124" s="6" t="inlineStr">
+      <c r="F127" s="6" t="inlineStr">
         <is>
           <t>Water (lb/hr)</t>
         </is>
       </c>
-      <c r="G124" s="6" t="inlineStr">
+      <c r="G127" s="6" t="inlineStr">
         <is>
           <t>Brix %</t>
         </is>
       </c>
-      <c r="H124" s="6" t="inlineStr">
+      <c r="H127" s="6" t="inlineStr">
         <is>
           <t>Purity %</t>
         </is>
       </c>
-      <c r="I124" s="6" t="inlineStr">
+      <c r="I127" s="6" t="inlineStr">
         <is>
           <t>ft³/hr</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="8" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
         <is>
           <t>A Molasses (undiluted)</t>
         </is>
       </c>
-      <c r="B125" s="8" t="inlineStr">
+      <c r="B128" s="8" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C125" s="9" t="n">
+      <c r="C128" s="9" t="n">
         <v>119441.5738467068</v>
       </c>
-      <c r="D125" s="9" t="n">
+      <c r="D128" s="9" t="n">
         <v>97942.09055429955</v>
       </c>
-      <c r="E125" s="9" t="n">
+      <c r="E128" s="9" t="n">
         <v>55826.99161595074</v>
       </c>
-      <c r="F125" s="9" t="n">
+      <c r="F128" s="9" t="n">
         <v>21499.48329240721</v>
       </c>
-      <c r="G125" s="10" t="n">
+      <c r="G128" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="H125" s="10" t="n">
+      <c r="H128" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I125" s="9" t="n">
+      <c r="I128" s="9" t="n">
         <v>1343.558979194719</v>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="12" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="12" t="inlineStr">
         <is>
           <t>Dilution Water</t>
         </is>
       </c>
-      <c r="B126" s="12" t="inlineStr">
+      <c r="B129" s="12" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C126" s="13" t="n">
+      <c r="C129" s="13" t="n">
         <v>20475.69837372117</v>
       </c>
-      <c r="D126" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E126" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F126" s="13" t="n">
+      <c r="D129" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" s="13" t="n">
         <v>20475.69837372117</v>
       </c>
-      <c r="G126" s="12" t="inlineStr"/>
-      <c r="H126" s="12" t="inlineStr"/>
-      <c r="I126" s="12" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="inlineStr">
+      <c r="G129" s="12" t="inlineStr"/>
+      <c r="H129" s="12" t="inlineStr"/>
+      <c r="I129" s="12" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
         <is>
           <t>A Molasses (diluted)</t>
         </is>
       </c>
-      <c r="B127" s="8" t="inlineStr">
+      <c r="B130" s="8" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C127" s="9" t="n">
+      <c r="C130" s="9" t="n">
         <v>139917.2722204279</v>
       </c>
-      <c r="D127" s="9" t="n">
+      <c r="D130" s="9" t="n">
         <v>97942.09055429955</v>
       </c>
-      <c r="E127" s="9" t="n">
+      <c r="E130" s="9" t="n">
         <v>55826.99161595074</v>
       </c>
-      <c r="F127" s="9" t="n">
+      <c r="F130" s="9" t="n">
         <v>41975.18166612838</v>
       </c>
-      <c r="G127" s="10" t="n">
+      <c r="G130" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="H127" s="10" t="n">
+      <c r="H130" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I127" s="9" t="n">
+      <c r="I130" s="9" t="n">
         <v>1664.963338036791</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="17" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="17" t="inlineStr">
         <is>
           <t>Total In</t>
         </is>
       </c>
-      <c r="B128" s="17" t="inlineStr"/>
-      <c r="C128" s="16" t="n">
+      <c r="B131" s="17" t="inlineStr"/>
+      <c r="C131" s="16" t="n">
         <v>139917.2722204279</v>
       </c>
-      <c r="D128" s="16" t="n">
+      <c r="D131" s="16" t="n">
         <v>97942.09055429955</v>
       </c>
-      <c r="E128" s="16" t="n">
+      <c r="E131" s="16" t="n">
         <v>55826.99161595074</v>
       </c>
-      <c r="F128" s="16" t="n">
+      <c r="F131" s="16" t="n">
         <v>41975.18166612838</v>
       </c>
-      <c r="G128" s="17" t="inlineStr"/>
-      <c r="H128" s="17" t="inlineStr"/>
-      <c r="I128" s="17" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="17" t="inlineStr">
+      <c r="G131" s="17" t="inlineStr"/>
+      <c r="H131" s="17" t="inlineStr"/>
+      <c r="I131" s="17" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="inlineStr">
         <is>
           <t>Total Out</t>
         </is>
       </c>
-      <c r="B129" s="17" t="inlineStr"/>
-      <c r="C129" s="16" t="n">
+      <c r="B132" s="17" t="inlineStr"/>
+      <c r="C132" s="16" t="n">
         <v>139917.2722204279</v>
       </c>
-      <c r="D129" s="16" t="n">
+      <c r="D132" s="16" t="n">
         <v>97942.09055429955</v>
       </c>
-      <c r="E129" s="16" t="n">
+      <c r="E132" s="16" t="n">
         <v>55826.99161595074</v>
       </c>
-      <c r="F129" s="16" t="n">
+      <c r="F132" s="16" t="n">
         <v>41975.18166612838</v>
       </c>
-      <c r="G129" s="17" t="inlineStr"/>
-      <c r="H129" s="17" t="inlineStr"/>
-      <c r="I129" s="17" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="17" t="inlineStr">
+      <c r="G132" s="17" t="inlineStr"/>
+      <c r="H132" s="17" t="inlineStr"/>
+      <c r="I132" s="17" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="inlineStr">
         <is>
           <t>Net (In - Out)</t>
         </is>
       </c>
-      <c r="B130" s="17" t="inlineStr"/>
-      <c r="C130" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D130" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E130" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F130" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G130" s="17" t="inlineStr"/>
-      <c r="H130" s="17" t="inlineStr"/>
-      <c r="I130" s="17" t="inlineStr"/>
-    </row>
-    <row r="132" ht="17" customHeight="1">
-      <c r="A132" s="4" t="inlineStr">
+      <c r="B133" s="17" t="inlineStr"/>
+      <c r="C133" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" s="17" t="inlineStr"/>
+      <c r="H133" s="17" t="inlineStr"/>
+      <c r="I133" s="17" t="inlineStr"/>
+    </row>
+    <row r="135" ht="17" customHeight="1">
+      <c r="A135" s="4" t="inlineStr">
         <is>
           <t>GRAIN PANS  [Grain Pans]</t>
         </is>
       </c>
-      <c r="B132" s="5" t="n"/>
-      <c r="C132" s="5" t="n"/>
-      <c r="D132" s="5" t="n"/>
-      <c r="E132" s="5" t="n"/>
-      <c r="F132" s="5" t="n"/>
-      <c r="G132" s="5" t="n"/>
-      <c r="H132" s="5" t="n"/>
-      <c r="I132" s="5" t="n"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="6" t="inlineStr">
+      <c r="B135" s="5" t="n"/>
+      <c r="C135" s="5" t="n"/>
+      <c r="D135" s="5" t="n"/>
+      <c r="E135" s="5" t="n"/>
+      <c r="F135" s="5" t="n"/>
+      <c r="G135" s="5" t="n"/>
+      <c r="H135" s="5" t="n"/>
+      <c r="I135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B133" s="6" t="inlineStr">
+      <c r="B136" s="6" t="inlineStr">
         <is>
           <t>Dir</t>
         </is>
       </c>
-      <c r="C133" s="6" t="inlineStr">
+      <c r="C136" s="6" t="inlineStr">
         <is>
           <t>Flow (lb/hr)</t>
         </is>
       </c>
-      <c r="D133" s="6" t="inlineStr">
+      <c r="D136" s="6" t="inlineStr">
         <is>
           <t>Solids (lb/hr)</t>
         </is>
       </c>
-      <c r="E133" s="6" t="inlineStr">
+      <c r="E136" s="6" t="inlineStr">
         <is>
           <t>Pol (lb/hr)</t>
         </is>
       </c>
-      <c r="F133" s="6" t="inlineStr">
+      <c r="F136" s="6" t="inlineStr">
         <is>
           <t>Water (lb/hr)</t>
         </is>
       </c>
-      <c r="G133" s="6" t="inlineStr">
+      <c r="G136" s="6" t="inlineStr">
         <is>
           <t>Brix %</t>
         </is>
       </c>
-      <c r="H133" s="6" t="inlineStr">
+      <c r="H136" s="6" t="inlineStr">
         <is>
           <t>Purity %</t>
         </is>
       </c>
-      <c r="I133" s="6" t="inlineStr">
+      <c r="I136" s="6" t="inlineStr">
         <is>
           <t>ft³/hr</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="8" t="inlineStr">
+    <row r="137">
+      <c r="A137" s="8" t="inlineStr">
         <is>
           <t>Syrup</t>
         </is>
       </c>
-      <c r="B134" s="8" t="inlineStr">
+      <c r="B137" s="8" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C134" s="9" t="n">
+      <c r="C137" s="9" t="n">
         <v>1796.955403809414</v>
       </c>
-      <c r="D134" s="9" t="n">
+      <c r="D137" s="9" t="n">
         <v>1084.688012476119</v>
       </c>
-      <c r="E134" s="9" t="n">
+      <c r="E137" s="9" t="n">
         <v>846.0566497313728</v>
       </c>
-      <c r="F134" s="9" t="n">
+      <c r="F137" s="9" t="n">
         <v>712.2673913332949</v>
       </c>
-      <c r="G134" s="10" t="n">
+      <c r="G137" s="10" t="n">
         <v>60.36254490103983</v>
       </c>
-      <c r="H134" s="10" t="n">
+      <c r="H137" s="10" t="n">
         <v>77.99999999999999</v>
       </c>
-      <c r="I134" s="9" t="n">
+      <c r="I137" s="9" t="n">
         <v>22.35609091760539</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="12" t="inlineStr">
+    <row r="138">
+      <c r="A138" s="12" t="inlineStr">
         <is>
           <t>A Molasses</t>
         </is>
       </c>
-      <c r="B135" s="12" t="inlineStr">
+      <c r="B138" s="12" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C135" s="13" t="n">
+      <c r="C138" s="13" t="n">
         <v>4197.518166612837</v>
       </c>
-      <c r="D135" s="13" t="n">
+      <c r="D138" s="13" t="n">
         <v>2938.262716628986</v>
       </c>
-      <c r="E135" s="13" t="n">
+      <c r="E138" s="13" t="n">
         <v>1674.809748478522</v>
       </c>
-      <c r="F135" s="13" t="n">
+      <c r="F138" s="13" t="n">
         <v>1259.255449983852</v>
       </c>
-      <c r="G135" s="14" t="n">
+      <c r="G138" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="H135" s="14" t="n">
+      <c r="H138" s="14" t="n">
         <v>57</v>
       </c>
-      <c r="I135" s="13" t="n">
+      <c r="I138" s="13" t="n">
         <v>49.94890014110372</v>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="8" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="8" t="inlineStr">
         <is>
           <t>Massecuite Out</t>
         </is>
       </c>
-      <c r="B136" s="8" t="inlineStr">
+      <c r="B139" s="8" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C136" s="9" t="n">
+      <c r="C139" s="9" t="n">
         <v>4571.534919437619</v>
       </c>
-      <c r="D136" s="9" t="n">
+      <c r="D139" s="9" t="n">
         <v>4022.950729105105</v>
       </c>
-      <c r="E136" s="9" t="n">
+      <c r="E139" s="9" t="n">
         <v>2520.866398209895</v>
       </c>
-      <c r="F136" s="9" t="n">
+      <c r="F139" s="9" t="n">
         <v>548.5841903325145</v>
       </c>
-      <c r="G136" s="10" t="n">
+      <c r="G139" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="H136" s="10" t="n">
+      <c r="H139" s="10" t="n">
         <v>62.66212459357301</v>
       </c>
-      <c r="I136" s="9" t="n">
+      <c r="I139" s="9" t="n">
         <v>49.98544669828643</v>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="12" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="12" t="inlineStr">
         <is>
           <t>Evaporated Water</t>
         </is>
       </c>
-      <c r="B137" s="12" t="inlineStr">
+      <c r="B140" s="12" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C137" s="13" t="n">
+      <c r="C140" s="13" t="n">
         <v>1422.938650984632</v>
       </c>
-      <c r="D137" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E137" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F137" s="13" t="n">
+      <c r="D140" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" s="13" t="n">
         <v>1422.938650984632</v>
       </c>
-      <c r="G137" s="12" t="inlineStr"/>
-      <c r="H137" s="12" t="inlineStr"/>
-      <c r="I137" s="12" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="17" t="inlineStr">
+      <c r="G140" s="12" t="inlineStr"/>
+      <c r="H140" s="12" t="inlineStr"/>
+      <c r="I140" s="12" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="inlineStr">
         <is>
           <t>Total In</t>
         </is>
       </c>
-      <c r="B138" s="17" t="inlineStr"/>
-      <c r="C138" s="16" t="n">
+      <c r="B141" s="17" t="inlineStr"/>
+      <c r="C141" s="16" t="n">
         <v>5994.473570422251</v>
       </c>
-      <c r="D138" s="16" t="n">
+      <c r="D141" s="16" t="n">
         <v>4022.950729105105</v>
       </c>
-      <c r="E138" s="16" t="n">
+      <c r="E141" s="16" t="n">
         <v>2520.866398209895</v>
       </c>
-      <c r="F138" s="16" t="n">
+      <c r="F141" s="16" t="n">
         <v>1971.522841317146</v>
       </c>
-      <c r="G138" s="17" t="inlineStr"/>
-      <c r="H138" s="17" t="inlineStr"/>
-      <c r="I138" s="17" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="17" t="inlineStr">
+      <c r="G141" s="17" t="inlineStr"/>
+      <c r="H141" s="17" t="inlineStr"/>
+      <c r="I141" s="17" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="inlineStr">
         <is>
           <t>Total Out</t>
         </is>
       </c>
-      <c r="B139" s="17" t="inlineStr"/>
-      <c r="C139" s="16" t="n">
+      <c r="B142" s="17" t="inlineStr"/>
+      <c r="C142" s="16" t="n">
         <v>5994.473570422251</v>
       </c>
-      <c r="D139" s="16" t="n">
+      <c r="D142" s="16" t="n">
         <v>4022.950729105105</v>
       </c>
-      <c r="E139" s="16" t="n">
+      <c r="E142" s="16" t="n">
         <v>2520.866398209895</v>
       </c>
-      <c r="F139" s="16" t="n">
+      <c r="F142" s="16" t="n">
         <v>1971.522841317146</v>
       </c>
-      <c r="G139" s="17" t="inlineStr"/>
-      <c r="H139" s="17" t="inlineStr"/>
-      <c r="I139" s="17" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="17" t="inlineStr">
+      <c r="G142" s="17" t="inlineStr"/>
+      <c r="H142" s="17" t="inlineStr"/>
+      <c r="I142" s="17" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="17" t="inlineStr">
         <is>
           <t>Net (In - Out)</t>
         </is>
       </c>
-      <c r="B140" s="17" t="inlineStr"/>
-      <c r="C140" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D140" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E140" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F140" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G140" s="17" t="inlineStr"/>
-      <c r="H140" s="17" t="inlineStr"/>
-      <c r="I140" s="17" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="18" t="inlineStr">
+      <c r="B143" s="17" t="inlineStr"/>
+      <c r="C143" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="17" t="inlineStr"/>
+      <c r="H143" s="17" t="inlineStr"/>
+      <c r="I143" s="17" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="18" t="inlineStr">
         <is>
           <t>Calandria steam type</t>
         </is>
       </c>
-      <c r="B141" s="18" t="inlineStr">
+      <c r="B144" s="18" t="inlineStr">
         <is>
           <t>Exhaust</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="18" t="inlineStr">
+    <row r="145">
+      <c r="A145" s="18" t="inlineStr">
         <is>
           <t>Calandria pressure</t>
         </is>
       </c>
-      <c r="B142" s="21" t="n">
+      <c r="B145" s="21" t="n">
         <v>29.696</v>
       </c>
-      <c r="C142" s="20" t="inlineStr">
+      <c r="C145" s="20" t="inlineStr">
         <is>
           <t>psia</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="18" t="inlineStr">
+    <row r="146">
+      <c r="A146" s="18" t="inlineStr">
         <is>
           <t>Calandria steam flow</t>
         </is>
       </c>
-      <c r="B143" s="22" t="n">
+      <c r="B146" s="22" t="n">
         <v>1713.311117829141</v>
       </c>
-      <c r="C143" s="20" t="inlineStr">
+      <c r="C146" s="20" t="inlineStr">
         <is>
           <t>lb/hr</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="17" customHeight="1">
-      <c r="A145" s="4" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="18" t="inlineStr">
+        <is>
+          <t>Heating surface</t>
+        </is>
+      </c>
+      <c r="B147" s="22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C147" s="20" t="inlineStr">
+        <is>
+          <t>ft²</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="18" t="inlineStr">
+        <is>
+          <t>dT (calandria - masse)</t>
+        </is>
+      </c>
+      <c r="B148" s="23" t="n">
+        <v>73.61757001819677</v>
+      </c>
+      <c r="C148" s="20" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="18" t="inlineStr">
+        <is>
+          <t>Overall U (back-calc)</t>
+        </is>
+      </c>
+      <c r="B149" s="23" t="n">
+        <v>7.33613909246579</v>
+      </c>
+      <c r="C149" s="20" t="inlineStr">
+        <is>
+          <t>BTU/hr·ft²·°F</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="17" customHeight="1">
+      <c r="A151" s="4" t="inlineStr">
         <is>
           <t>C PANS  [C Pans]</t>
         </is>
       </c>
-      <c r="B145" s="5" t="n"/>
-      <c r="C145" s="5" t="n"/>
-      <c r="D145" s="5" t="n"/>
-      <c r="E145" s="5" t="n"/>
-      <c r="F145" s="5" t="n"/>
-      <c r="G145" s="5" t="n"/>
-      <c r="H145" s="5" t="n"/>
-      <c r="I145" s="5" t="n"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="6" t="inlineStr">
+      <c r="B151" s="5" t="n"/>
+      <c r="C151" s="5" t="n"/>
+      <c r="D151" s="5" t="n"/>
+      <c r="E151" s="5" t="n"/>
+      <c r="F151" s="5" t="n"/>
+      <c r="G151" s="5" t="n"/>
+      <c r="H151" s="5" t="n"/>
+      <c r="I151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="6" t="inlineStr">
         <is>
           <t>Stream</t>
         </is>
       </c>
-      <c r="B146" s="6" t="inlineStr">
+      <c r="B152" s="6" t="inlineStr">
         <is>
           <t>Dir</t>
         </is>
       </c>
-      <c r="C146" s="6" t="inlineStr">
+      <c r="C152" s="6" t="inlineStr">
         <is>
           <t>Flow (lb/hr)</t>
         </is>
       </c>
-      <c r="D146" s="6" t="inlineStr">
+      <c r="D152" s="6" t="inlineStr">
         <is>
           <t>Solids (lb/hr)</t>
         </is>
       </c>
-      <c r="E146" s="6" t="inlineStr">
+      <c r="E152" s="6" t="inlineStr">
         <is>
           <t>Pol (lb/hr)</t>
         </is>
       </c>
-      <c r="F146" s="6" t="inlineStr">
+      <c r="F152" s="6" t="inlineStr">
         <is>
           <t>Water (lb/hr)</t>
         </is>
       </c>
-      <c r="G146" s="6" t="inlineStr">
+      <c r="G152" s="6" t="inlineStr">
         <is>
           <t>Brix %</t>
         </is>
       </c>
-      <c r="H146" s="6" t="inlineStr">
+      <c r="H152" s="6" t="inlineStr">
         <is>
           <t>Purity %</t>
         </is>
       </c>
-      <c r="I146" s="6" t="inlineStr">
+      <c r="I152" s="6" t="inlineStr">
         <is>
           <t>ft³/hr</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="8" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="8" t="inlineStr">
         <is>
           <t>Grain Massecuite</t>
         </is>
       </c>
-      <c r="B147" s="8" t="inlineStr">
+      <c r="B153" s="8" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C147" s="9" t="n">
+      <c r="C153" s="9" t="n">
         <v>4571.534919437619</v>
       </c>
-      <c r="D147" s="9" t="n">
+      <c r="D153" s="9" t="n">
         <v>4022.950729105105</v>
       </c>
-      <c r="E147" s="9" t="n">
+      <c r="E153" s="9" t="n">
         <v>2520.866398209895</v>
       </c>
-      <c r="F147" s="9" t="n">
+      <c r="F153" s="9" t="n">
         <v>548.584190332514</v>
       </c>
-      <c r="G147" s="10" t="n">
+      <c r="G153" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="H147" s="10" t="n">
+      <c r="H153" s="10" t="n">
         <v>62.66212459357301</v>
       </c>
-      <c r="I147" s="9" t="n">
+      <c r="I153" s="9" t="n">
         <v>49.98544669828643</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="12" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
         <is>
           <t>A Molasses</t>
         </is>
       </c>
-      <c r="B148" s="12" t="inlineStr">
+      <c r="B154" s="12" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C148" s="13" t="n">
+      <c r="C154" s="13" t="n">
         <v>93744.57238768671</v>
       </c>
-      <c r="D148" s="13" t="n">
+      <c r="D154" s="13" t="n">
         <v>65621.20067138071</v>
       </c>
-      <c r="E148" s="13" t="n">
+      <c r="E154" s="13" t="n">
         <v>37404.084382687</v>
       </c>
-      <c r="F148" s="13" t="n">
+      <c r="F154" s="13" t="n">
         <v>28123.37171630601</v>
       </c>
-      <c r="G148" s="14" t="n">
+      <c r="G154" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="H148" s="14" t="n">
+      <c r="H154" s="14" t="n">
         <v>57</v>
       </c>
-      <c r="I148" s="13" t="n">
+      <c r="I154" s="13" t="n">
         <v>1115.52543648465</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="8" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="8" t="inlineStr">
         <is>
           <t>Syrup</t>
         </is>
       </c>
-      <c r="B149" s="8" t="inlineStr">
+      <c r="B155" s="8" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C149" s="9" t="n">
+      <c r="C155" s="9" t="n">
         <v>8984.777019047069</v>
       </c>
-      <c r="D149" s="9" t="n">
+      <c r="D155" s="9" t="n">
         <v>5423.440062380595</v>
       </c>
-      <c r="E149" s="9" t="n">
+      <c r="E155" s="9" t="n">
         <v>4230.283248656863</v>
       </c>
-      <c r="F149" s="9" t="n">
+      <c r="F155" s="9" t="n">
         <v>3561.336956666474</v>
       </c>
-      <c r="G149" s="10" t="n">
+      <c r="G155" s="10" t="n">
         <v>60.36254490103983</v>
       </c>
-      <c r="H149" s="10" t="n">
+      <c r="H155" s="10" t="n">
         <v>77.99999999999999</v>
       </c>
-      <c r="I149" s="9" t="n">
+      <c r="I155" s="9" t="n">
         <v>111.7804545880269</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="12" t="inlineStr">
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
         <is>
           <t>Massecuite Out</t>
         </is>
       </c>
-      <c r="B150" s="12" t="inlineStr">
+      <c r="B156" s="12" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C150" s="13" t="n">
+      <c r="C156" s="13" t="n">
         <v>78604.80781451979</v>
       </c>
-      <c r="D150" s="13" t="n">
+      <c r="D156" s="13" t="n">
         <v>75067.5914628664</v>
       </c>
-      <c r="E150" s="13" t="n">
+      <c r="E156" s="13" t="n">
         <v>44155.23402955376</v>
       </c>
-      <c r="F150" s="13" t="n">
+      <c r="F156" s="13" t="n">
         <v>3537.216351653391</v>
       </c>
-      <c r="G150" s="14" t="n">
+      <c r="G156" s="14" t="n">
         <v>95.5</v>
       </c>
-      <c r="H150" s="14" t="n">
+      <c r="H156" s="14" t="n">
         <v>58.82063506912431</v>
       </c>
-      <c r="I150" s="13" t="n">
+      <c r="I156" s="13" t="n">
         <v>829.4290410571672</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="8" t="inlineStr">
+    <row r="157">
+      <c r="A157" s="8" t="inlineStr">
         <is>
           <t>Evaporated Water</t>
         </is>
       </c>
-      <c r="B151" s="8" t="inlineStr">
+      <c r="B157" s="8" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C151" s="9" t="n">
+      <c r="C157" s="9" t="n">
         <v>28696.07651165161</v>
       </c>
-      <c r="D151" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E151" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F151" s="9" t="n">
+      <c r="D157" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="9" t="n">
         <v>28696.07651165161</v>
       </c>
-      <c r="G151" s="8" t="inlineStr"/>
-      <c r="H151" s="8" t="inlineStr"/>
-      <c r="I151" s="8" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="17" t="inlineStr">
+      <c r="G157" s="8" t="inlineStr"/>
+      <c r="H157" s="8" t="inlineStr"/>
+      <c r="I157" s="8" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="17" t="inlineStr">
         <is>
           <t>Total In</t>
         </is>
       </c>
-      <c r="B152" s="17" t="inlineStr"/>
-      <c r="C152" s="16" t="n">
+      <c r="B158" s="17" t="inlineStr"/>
+      <c r="C158" s="16" t="n">
         <v>107300.8843261714</v>
       </c>
-      <c r="D152" s="16" t="n">
+      <c r="D158" s="16" t="n">
         <v>75067.5914628664</v>
       </c>
-      <c r="E152" s="16" t="n">
+      <c r="E158" s="16" t="n">
         <v>44155.23402955376</v>
       </c>
-      <c r="F152" s="16" t="n">
+      <c r="F158" s="16" t="n">
         <v>32233.292863305</v>
       </c>
-      <c r="G152" s="17" t="inlineStr"/>
-      <c r="H152" s="17" t="inlineStr"/>
-      <c r="I152" s="17" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="17" t="inlineStr">
+      <c r="G158" s="17" t="inlineStr"/>
+      <c r="H158" s="17" t="inlineStr"/>
+      <c r="I158" s="17" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="17" t="inlineStr">
         <is>
           <t>Total Out</t>
         </is>
       </c>
-      <c r="B153" s="17" t="inlineStr"/>
-      <c r="C153" s="16" t="n">
+      <c r="B159" s="17" t="inlineStr"/>
+      <c r="C159" s="16" t="n">
         <v>107300.8843261714</v>
       </c>
-      <c r="D153" s="16" t="n">
+      <c r="D159" s="16" t="n">
         <v>75067.5914628664</v>
       </c>
-      <c r="E153" s="16" t="n">
+      <c r="E159" s="16" t="n">
         <v>44155.23402955376</v>
       </c>
-      <c r="F153" s="16" t="n">
+      <c r="F159" s="16" t="n">
         <v>32233.292863305</v>
       </c>
-      <c r="G153" s="17" t="inlineStr"/>
-      <c r="H153" s="17" t="inlineStr"/>
-      <c r="I153" s="17" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="17" t="inlineStr">
+      <c r="G159" s="17" t="inlineStr"/>
+      <c r="H159" s="17" t="inlineStr"/>
+      <c r="I159" s="17" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="17" t="inlineStr">
         <is>
           <t>Net (In - Out)</t>
         </is>
       </c>
-      <c r="B154" s="17" t="inlineStr"/>
-      <c r="C154" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D154" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E154" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F154" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" s="17" t="inlineStr"/>
-      <c r="H154" s="17" t="inlineStr"/>
-      <c r="I154" s="17" t="inlineStr"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="18" t="inlineStr">
+      <c r="B160" s="17" t="inlineStr"/>
+      <c r="C160" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D160" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" s="17" t="inlineStr"/>
+      <c r="H160" s="17" t="inlineStr"/>
+      <c r="I160" s="17" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="18" t="inlineStr">
         <is>
           <t>Calandria steam type</t>
         </is>
       </c>
-      <c r="B155" s="18" t="inlineStr">
+      <c r="B161" s="18" t="inlineStr">
         <is>
           <t>Exhaust</t>
         </is>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="18" t="inlineStr">
+    <row r="162">
+      <c r="A162" s="18" t="inlineStr">
         <is>
           <t>Calandria pressure</t>
         </is>
       </c>
-      <c r="B156" s="21" t="n">
+      <c r="B162" s="21" t="n">
         <v>21.696</v>
       </c>
-      <c r="C156" s="20" t="inlineStr">
+      <c r="C162" s="20" t="inlineStr">
         <is>
           <t>psia</t>
         </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="18" t="inlineStr">
-        <is>
-          <t>Calandria steam flow</t>
-        </is>
-      </c>
-      <c r="B157" s="22" t="n">
-        <v>33672.02372451993</v>
-      </c>
-      <c r="C157" s="20" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" ht="17" customHeight="1">
-      <c r="A159" s="4" t="inlineStr">
-        <is>
-          <t>C CRYSTALLIZERS  [C Crystallizers]</t>
-        </is>
-      </c>
-      <c r="B159" s="5" t="n"/>
-      <c r="C159" s="5" t="n"/>
-      <c r="D159" s="5" t="n"/>
-      <c r="E159" s="5" t="n"/>
-      <c r="F159" s="5" t="n"/>
-      <c r="G159" s="5" t="n"/>
-      <c r="H159" s="5" t="n"/>
-      <c r="I159" s="5" t="n"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="6" t="inlineStr">
-        <is>
-          <t>Stream</t>
-        </is>
-      </c>
-      <c r="B160" s="6" t="inlineStr">
-        <is>
-          <t>Dir</t>
-        </is>
-      </c>
-      <c r="C160" s="6" t="inlineStr">
-        <is>
-          <t>Flow (lb/hr)</t>
-        </is>
-      </c>
-      <c r="D160" s="6" t="inlineStr">
-        <is>
-          <t>Solids (lb/hr)</t>
-        </is>
-      </c>
-      <c r="E160" s="6" t="inlineStr">
-        <is>
-          <t>Pol (lb/hr)</t>
-        </is>
-      </c>
-      <c r="F160" s="6" t="inlineStr">
-        <is>
-          <t>Water (lb/hr)</t>
-        </is>
-      </c>
-      <c r="G160" s="6" t="inlineStr">
-        <is>
-          <t>Brix %</t>
-        </is>
-      </c>
-      <c r="H160" s="6" t="inlineStr">
-        <is>
-          <t>Purity %</t>
-        </is>
-      </c>
-      <c r="I160" s="6" t="inlineStr">
-        <is>
-          <t>ft³/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="8" t="inlineStr">
-        <is>
-          <t>Massecuite In  (T=173.8 °F)</t>
-        </is>
-      </c>
-      <c r="B161" s="8" t="inlineStr">
-        <is>
-          <t>In</t>
-        </is>
-      </c>
-      <c r="C161" s="9" t="n">
-        <v>78604.80781451979</v>
-      </c>
-      <c r="D161" s="9" t="n">
-        <v>75067.5914628664</v>
-      </c>
-      <c r="E161" s="9" t="n">
-        <v>44155.23402955377</v>
-      </c>
-      <c r="F161" s="9" t="n">
-        <v>3537.216351653391</v>
-      </c>
-      <c r="G161" s="10" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="H161" s="10" t="n">
-        <v>58.82063506912431</v>
-      </c>
-      <c r="I161" s="9" t="n">
-        <v>829.4290410571672</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="12" t="inlineStr">
-        <is>
-          <t>Massecuite Out  (T=120.0 °F)</t>
-        </is>
-      </c>
-      <c r="B162" s="12" t="inlineStr">
-        <is>
-          <t>Out</t>
-        </is>
-      </c>
-      <c r="C162" s="13" t="n">
-        <v>78604.80781451979</v>
-      </c>
-      <c r="D162" s="13" t="n">
-        <v>75067.5914628664</v>
-      </c>
-      <c r="E162" s="13" t="n">
-        <v>44155.23402955377</v>
-      </c>
-      <c r="F162" s="13" t="n">
-        <v>3537.216351653391</v>
-      </c>
-      <c r="G162" s="14" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="H162" s="14" t="n">
-        <v>58.82063506912431</v>
-      </c>
-      <c r="I162" s="13" t="n">
-        <v>829.4290410571672</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="18" t="inlineStr">
         <is>
-          <t>ML purity in -&gt; out</t>
-        </is>
-      </c>
-      <c r="B163" s="18" t="inlineStr">
-        <is>
-          <t>30.0 -&gt; 30.0</t>
-        </is>
+          <t>Calandria steam flow</t>
+        </is>
+      </c>
+      <c r="B163" s="22" t="n">
+        <v>33672.02372451993</v>
       </c>
       <c r="C163" s="20" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>lb/hr</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="18" t="inlineStr">
         <is>
-          <t>Crystal content in -&gt; out</t>
-        </is>
-      </c>
-      <c r="B164" s="18" t="inlineStr">
-        <is>
-          <t>39.3 -&gt; 39.3</t>
-        </is>
+          <t>Heating surface</t>
+        </is>
+      </c>
+      <c r="B164" s="22" t="n">
+        <v>12000</v>
       </c>
       <c r="C164" s="20" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>ft²</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="18" t="inlineStr">
         <is>
-          <t>Duty</t>
-        </is>
-      </c>
-      <c r="B165" s="22" t="n">
-        <v>1930652.761039244</v>
+          <t>dT (calandria - masse)</t>
+        </is>
+      </c>
+      <c r="B165" s="23" t="n">
+        <v>58.46505960826261</v>
       </c>
       <c r="C165" s="20" t="inlineStr">
         <is>
-          <t>BTU/hr</t>
+          <t>°F</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="18" t="inlineStr">
         <is>
-          <t>Cooling Water</t>
-        </is>
-      </c>
-      <c r="B166" s="22" t="n">
-        <v>96532.63805196219</v>
+          <t>Overall U (back-calc)</t>
+        </is>
+      </c>
+      <c r="B166" s="23" t="n">
+        <v>45.93560552103934</v>
       </c>
       <c r="C166" s="20" t="inlineStr">
         <is>
-          <t>lb/hr  (193 gpm, 85 -&gt; 105 °F)</t>
+          <t>BTU/hr·ft²·°F</t>
         </is>
       </c>
     </row>
     <row r="168" ht="17" customHeight="1">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>C REHEATERS  [C Reheaters]</t>
+          <t>C CRYSTALLIZERS  [C Crystallizers]</t>
         </is>
       </c>
       <c r="B168" s="5" t="n"/>
@@ -3392,7 +3335,7 @@
     <row r="170">
       <c r="A170" s="8" t="inlineStr">
         <is>
-          <t>Massecuite In  (T=120.0 °F)</t>
+          <t>Massecuite In  (T=173.8 °F)</t>
         </is>
       </c>
       <c r="B170" s="8" t="inlineStr">
@@ -3425,7 +3368,7 @@
     <row r="171">
       <c r="A171" s="12" t="inlineStr">
         <is>
-          <t>Massecuite Out  (T=130.0 °F)</t>
+          <t>Massecuite Out  (T=120.0 °F)</t>
         </is>
       </c>
       <c r="B171" s="12" t="inlineStr">
@@ -3496,7 +3439,7 @@
         </is>
       </c>
       <c r="B174" s="22" t="n">
-        <v>358636.0077499028</v>
+        <v>1930652.761039244</v>
       </c>
       <c r="C174" s="20" t="inlineStr">
         <is>
@@ -3507,22 +3450,22 @@
     <row r="175">
       <c r="A175" s="18" t="inlineStr">
         <is>
-          <t>Hot Water</t>
+          <t>Cooling Water</t>
         </is>
       </c>
       <c r="B175" s="22" t="n">
-        <v>23909.06718332686</v>
+        <v>96532.63805196219</v>
       </c>
       <c r="C175" s="20" t="inlineStr">
         <is>
-          <t>lb/hr  (48 gpm, 150 -&gt; 135 °F)</t>
+          <t>lb/hr  (193 gpm, 85 -&gt; 105 °F)</t>
         </is>
       </c>
     </row>
     <row r="177" ht="17" customHeight="1">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>C CENTRIFUGALS  [C Centrifugals]</t>
+          <t>C REHEATERS  [C Reheaters]</t>
         </is>
       </c>
       <c r="B177" s="5" t="n"/>
@@ -3584,7 +3527,7 @@
     <row r="179">
       <c r="A179" s="8" t="inlineStr">
         <is>
-          <t>Massecuite</t>
+          <t>Massecuite In  (T=120.0 °F)</t>
         </is>
       </c>
       <c r="B179" s="8" t="inlineStr">
@@ -3617,318 +3560,286 @@
     <row r="180">
       <c r="A180" s="12" t="inlineStr">
         <is>
+          <t>Massecuite Out  (T=130.0 °F)</t>
+        </is>
+      </c>
+      <c r="B180" s="12" t="inlineStr">
+        <is>
+          <t>Out</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="n">
+        <v>78604.80781451979</v>
+      </c>
+      <c r="D180" s="13" t="n">
+        <v>75067.5914628664</v>
+      </c>
+      <c r="E180" s="13" t="n">
+        <v>44155.23402955377</v>
+      </c>
+      <c r="F180" s="13" t="n">
+        <v>3537.216351653391</v>
+      </c>
+      <c r="G180" s="14" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="H180" s="14" t="n">
+        <v>58.82063506912431</v>
+      </c>
+      <c r="I180" s="13" t="n">
+        <v>829.4290410571672</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="18" t="inlineStr">
+        <is>
+          <t>ML purity in -&gt; out</t>
+        </is>
+      </c>
+      <c r="B181" s="18" t="inlineStr">
+        <is>
+          <t>30.0 -&gt; 30.0</t>
+        </is>
+      </c>
+      <c r="C181" s="20" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="18" t="inlineStr">
+        <is>
+          <t>Crystal content in -&gt; out</t>
+        </is>
+      </c>
+      <c r="B182" s="18" t="inlineStr">
+        <is>
+          <t>39.3 -&gt; 39.3</t>
+        </is>
+      </c>
+      <c r="C182" s="20" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="18" t="inlineStr">
+        <is>
+          <t>Duty</t>
+        </is>
+      </c>
+      <c r="B183" s="22" t="n">
+        <v>358636.0077499028</v>
+      </c>
+      <c r="C183" s="20" t="inlineStr">
+        <is>
+          <t>BTU/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="18" t="inlineStr">
+        <is>
+          <t>Hot Water</t>
+        </is>
+      </c>
+      <c r="B184" s="22" t="n">
+        <v>23909.06718332686</v>
+      </c>
+      <c r="C184" s="20" t="inlineStr">
+        <is>
+          <t>lb/hr  (48 gpm, 150 -&gt; 135 °F)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="17" customHeight="1">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>C CENTRIFUGALS  [C Centrifugals]</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="n"/>
+      <c r="C186" s="5" t="n"/>
+      <c r="D186" s="5" t="n"/>
+      <c r="E186" s="5" t="n"/>
+      <c r="F186" s="5" t="n"/>
+      <c r="G186" s="5" t="n"/>
+      <c r="H186" s="5" t="n"/>
+      <c r="I186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="6" t="inlineStr">
+        <is>
+          <t>Stream</t>
+        </is>
+      </c>
+      <c r="B187" s="6" t="inlineStr">
+        <is>
+          <t>Dir</t>
+        </is>
+      </c>
+      <c r="C187" s="6" t="inlineStr">
+        <is>
+          <t>Flow (lb/hr)</t>
+        </is>
+      </c>
+      <c r="D187" s="6" t="inlineStr">
+        <is>
+          <t>Solids (lb/hr)</t>
+        </is>
+      </c>
+      <c r="E187" s="6" t="inlineStr">
+        <is>
+          <t>Pol (lb/hr)</t>
+        </is>
+      </c>
+      <c r="F187" s="6" t="inlineStr">
+        <is>
+          <t>Water (lb/hr)</t>
+        </is>
+      </c>
+      <c r="G187" s="6" t="inlineStr">
+        <is>
+          <t>Brix %</t>
+        </is>
+      </c>
+      <c r="H187" s="6" t="inlineStr">
+        <is>
+          <t>Purity %</t>
+        </is>
+      </c>
+      <c r="I187" s="6" t="inlineStr">
+        <is>
+          <t>ft³/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="8" t="inlineStr">
+        <is>
+          <t>Massecuite</t>
+        </is>
+      </c>
+      <c r="B188" s="8" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="C188" s="9" t="n">
+        <v>78604.80781451979</v>
+      </c>
+      <c r="D188" s="9" t="n">
+        <v>75067.5914628664</v>
+      </c>
+      <c r="E188" s="9" t="n">
+        <v>44155.23402955377</v>
+      </c>
+      <c r="F188" s="9" t="n">
+        <v>3537.216351653391</v>
+      </c>
+      <c r="G188" s="10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="H188" s="10" t="n">
+        <v>58.82063506912431</v>
+      </c>
+      <c r="I188" s="9" t="n">
+        <v>829.4290410571672</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="12" t="inlineStr">
+        <is>
           <t>Wash Water</t>
         </is>
       </c>
-      <c r="B180" s="12" t="inlineStr">
+      <c r="B189" s="12" t="inlineStr">
         <is>
           <t>In</t>
         </is>
       </c>
-      <c r="C180" s="13" t="n">
+      <c r="C189" s="13" t="n">
         <v>5874.303955508396</v>
       </c>
-      <c r="D180" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E180" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F180" s="13" t="n">
+      <c r="D189" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E189" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" s="13" t="n">
         <v>5874.303955508396</v>
       </c>
-      <c r="G180" s="12" t="inlineStr"/>
-      <c r="H180" s="12" t="inlineStr"/>
-      <c r="I180" s="12" t="inlineStr"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="8" t="inlineStr">
+      <c r="G189" s="12" t="inlineStr"/>
+      <c r="H189" s="12" t="inlineStr"/>
+      <c r="I189" s="12" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="8" t="inlineStr">
         <is>
           <t>Sugar Out</t>
         </is>
       </c>
-      <c r="B181" s="8" t="inlineStr">
+      <c r="B190" s="8" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C181" s="9" t="n">
+      <c r="C190" s="9" t="n">
         <v>44574.76778033299</v>
       </c>
-      <c r="D181" s="9" t="n">
+      <c r="D190" s="9" t="n">
         <v>42346.02939131634</v>
       </c>
-      <c r="E181" s="9" t="n">
+      <c r="E190" s="9" t="n">
         <v>33029.90292522674</v>
       </c>
-      <c r="F181" s="9" t="n">
+      <c r="F190" s="9" t="n">
         <v>2228.738389016653</v>
       </c>
-      <c r="G181" s="10" t="n">
+      <c r="G190" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="H181" s="10" t="n">
+      <c r="H190" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I181" s="9" t="n">
+      <c r="I190" s="9" t="n">
         <v>471.4659015221285</v>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="12" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="12" t="inlineStr">
         <is>
           <t>Molasses Out</t>
         </is>
       </c>
-      <c r="B182" s="12" t="inlineStr">
+      <c r="B191" s="12" t="inlineStr">
         <is>
           <t>Out</t>
         </is>
       </c>
-      <c r="C182" s="13" t="n">
+      <c r="C191" s="13" t="n">
         <v>39904.3439896952</v>
       </c>
-      <c r="D182" s="13" t="n">
+      <c r="D191" s="13" t="n">
         <v>32721.56207155007</v>
       </c>
-      <c r="E182" s="13" t="n">
+      <c r="E191" s="13" t="n">
         <v>11125.33110432702</v>
       </c>
-      <c r="F182" s="13" t="n">
+      <c r="F191" s="13" t="n">
         <v>7182.781918145134</v>
       </c>
-      <c r="G182" s="14" t="n">
+      <c r="G191" s="14" t="n">
         <v>82</v>
       </c>
-      <c r="H182" s="14" t="n">
+      <c r="H191" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="I182" s="13" t="n">
+      <c r="I191" s="13" t="n">
         <v>448.8708407764174</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="17" t="inlineStr">
-        <is>
-          <t>Total In</t>
-        </is>
-      </c>
-      <c r="B183" s="17" t="inlineStr"/>
-      <c r="C183" s="16" t="n">
-        <v>84479.11177002819</v>
-      </c>
-      <c r="D183" s="16" t="n">
-        <v>75067.5914628664</v>
-      </c>
-      <c r="E183" s="16" t="n">
-        <v>44155.23402955377</v>
-      </c>
-      <c r="F183" s="16" t="n">
-        <v>9411.520307161787</v>
-      </c>
-      <c r="G183" s="17" t="inlineStr"/>
-      <c r="H183" s="17" t="inlineStr"/>
-      <c r="I183" s="17" t="inlineStr"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="17" t="inlineStr">
-        <is>
-          <t>Total Out</t>
-        </is>
-      </c>
-      <c r="B184" s="17" t="inlineStr"/>
-      <c r="C184" s="16" t="n">
-        <v>84479.11177002819</v>
-      </c>
-      <c r="D184" s="16" t="n">
-        <v>75067.5914628664</v>
-      </c>
-      <c r="E184" s="16" t="n">
-        <v>44155.23402955377</v>
-      </c>
-      <c r="F184" s="16" t="n">
-        <v>9411.520307161787</v>
-      </c>
-      <c r="G184" s="17" t="inlineStr"/>
-      <c r="H184" s="17" t="inlineStr"/>
-      <c r="I184" s="17" t="inlineStr"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="17" t="inlineStr">
-        <is>
-          <t>Net (In - Out)</t>
-        </is>
-      </c>
-      <c r="B185" s="17" t="inlineStr"/>
-      <c r="C185" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D185" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E185" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F185" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G185" s="17" t="inlineStr"/>
-      <c r="H185" s="17" t="inlineStr"/>
-      <c r="I185" s="17" t="inlineStr"/>
-    </row>
-    <row r="187" ht="17" customHeight="1">
-      <c r="A187" s="4" t="inlineStr">
-        <is>
-          <t>C MAGMA  (mingler target 92.0 Bx)</t>
-        </is>
-      </c>
-      <c r="B187" s="5" t="n"/>
-      <c r="C187" s="5" t="n"/>
-      <c r="D187" s="5" t="n"/>
-      <c r="E187" s="5" t="n"/>
-      <c r="F187" s="5" t="n"/>
-      <c r="G187" s="5" t="n"/>
-      <c r="H187" s="5" t="n"/>
-      <c r="I187" s="5" t="n"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="6" t="inlineStr">
-        <is>
-          <t>Stream</t>
-        </is>
-      </c>
-      <c r="B188" s="6" t="inlineStr">
-        <is>
-          <t>Dir</t>
-        </is>
-      </c>
-      <c r="C188" s="6" t="inlineStr">
-        <is>
-          <t>Flow (lb/hr)</t>
-        </is>
-      </c>
-      <c r="D188" s="6" t="inlineStr">
-        <is>
-          <t>Solids (lb/hr)</t>
-        </is>
-      </c>
-      <c r="E188" s="6" t="inlineStr">
-        <is>
-          <t>Pol (lb/hr)</t>
-        </is>
-      </c>
-      <c r="F188" s="6" t="inlineStr">
-        <is>
-          <t>Water (lb/hr)</t>
-        </is>
-      </c>
-      <c r="G188" s="6" t="inlineStr">
-        <is>
-          <t>Brix %</t>
-        </is>
-      </c>
-      <c r="H188" s="6" t="inlineStr">
-        <is>
-          <t>Purity %</t>
-        </is>
-      </c>
-      <c r="I188" s="6" t="inlineStr">
-        <is>
-          <t>ft³/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="8" t="inlineStr">
-        <is>
-          <t>C Sugar</t>
-        </is>
-      </c>
-      <c r="B189" s="8" t="inlineStr">
-        <is>
-          <t>In</t>
-        </is>
-      </c>
-      <c r="C189" s="9" t="n">
-        <v>44574.76778033299</v>
-      </c>
-      <c r="D189" s="9" t="n">
-        <v>42346.02939131634</v>
-      </c>
-      <c r="E189" s="9" t="n">
-        <v>33029.90292522674</v>
-      </c>
-      <c r="F189" s="9" t="n">
-        <v>2228.738389016653</v>
-      </c>
-      <c r="G189" s="10" t="n">
-        <v>95</v>
-      </c>
-      <c r="H189" s="10" t="n">
-        <v>78</v>
-      </c>
-      <c r="I189" s="9" t="n">
-        <v>471.4659015221285</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="12" t="inlineStr">
-        <is>
-          <t>Mingler Water</t>
-        </is>
-      </c>
-      <c r="B190" s="12" t="inlineStr">
-        <is>
-          <t>In</t>
-        </is>
-      </c>
-      <c r="C190" s="13" t="n">
-        <v>1453.525036315201</v>
-      </c>
-      <c r="D190" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E190" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F190" s="13" t="n">
-        <v>1453.525036315201</v>
-      </c>
-      <c r="G190" s="12" t="inlineStr"/>
-      <c r="H190" s="12" t="inlineStr"/>
-      <c r="I190" s="12" t="inlineStr"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="8" t="inlineStr">
-        <is>
-          <t>C Magma</t>
-        </is>
-      </c>
-      <c r="B191" s="8" t="inlineStr">
-        <is>
-          <t>Out</t>
-        </is>
-      </c>
-      <c r="C191" s="9" t="n">
-        <v>46028.29281664819</v>
-      </c>
-      <c r="D191" s="9" t="n">
-        <v>42346.02939131634</v>
-      </c>
-      <c r="E191" s="9" t="n">
-        <v>33029.90292522674</v>
-      </c>
-      <c r="F191" s="9" t="n">
-        <v>3682.263425331854</v>
-      </c>
-      <c r="G191" s="10" t="n">
-        <v>92</v>
-      </c>
-      <c r="H191" s="10" t="n">
-        <v>78</v>
-      </c>
-      <c r="I191" s="9" t="n">
-        <v>493.821866009951</v>
       </c>
     </row>
     <row r="192">
@@ -3939,16 +3850,16 @@
       </c>
       <c r="B192" s="17" t="inlineStr"/>
       <c r="C192" s="16" t="n">
-        <v>46028.29281664819</v>
+        <v>84479.11177002819</v>
       </c>
       <c r="D192" s="16" t="n">
-        <v>42346.02939131634</v>
+        <v>75067.5914628664</v>
       </c>
       <c r="E192" s="16" t="n">
-        <v>33029.90292522674</v>
+        <v>44155.23402955377</v>
       </c>
       <c r="F192" s="16" t="n">
-        <v>3682.263425331854</v>
+        <v>9411.520307161787</v>
       </c>
       <c r="G192" s="17" t="inlineStr"/>
       <c r="H192" s="17" t="inlineStr"/>
@@ -3962,16 +3873,16 @@
       </c>
       <c r="B193" s="17" t="inlineStr"/>
       <c r="C193" s="16" t="n">
-        <v>46028.29281664819</v>
+        <v>84479.11177002819</v>
       </c>
       <c r="D193" s="16" t="n">
-        <v>42346.02939131634</v>
+        <v>75067.5914628664</v>
       </c>
       <c r="E193" s="16" t="n">
-        <v>33029.90292522674</v>
+        <v>44155.23402955377</v>
       </c>
       <c r="F193" s="16" t="n">
-        <v>3682.263425331854</v>
+        <v>9411.520307161787</v>
       </c>
       <c r="G193" s="17" t="inlineStr"/>
       <c r="H193" s="17" t="inlineStr"/>
@@ -4003,7 +3914,7 @@
     <row r="196" ht="17" customHeight="1">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>C MAGMA DISTRIBUTION</t>
+          <t>C MAGMA  (mingler target 92.0 Bx)</t>
         </is>
       </c>
       <c r="B196" s="5" t="n"/>
@@ -4065,7 +3976,7 @@
     <row r="198">
       <c r="A198" s="8" t="inlineStr">
         <is>
-          <t>Magma (total)</t>
+          <t>C Sugar</t>
         </is>
       </c>
       <c r="B198" s="8" t="inlineStr">
@@ -4074,7 +3985,7 @@
         </is>
       </c>
       <c r="C198" s="9" t="n">
-        <v>46028.29281664819</v>
+        <v>44574.76778033299</v>
       </c>
       <c r="D198" s="9" t="n">
         <v>42346.02939131634</v>
@@ -4083,55 +3994,49 @@
         <v>33029.90292522674</v>
       </c>
       <c r="F198" s="9" t="n">
-        <v>3682.263425331854</v>
+        <v>2228.738389016653</v>
       </c>
       <c r="G198" s="10" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H198" s="10" t="n">
         <v>78</v>
       </c>
       <c r="I198" s="9" t="n">
-        <v>493.821866009951</v>
+        <v>471.4659015221285</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="12" t="inlineStr">
         <is>
-          <t>C Magma to A Footing</t>
+          <t>Mingler Water</t>
         </is>
       </c>
       <c r="B199" s="12" t="inlineStr">
         <is>
-          <t>Out</t>
+          <t>In</t>
         </is>
       </c>
       <c r="C199" s="13" t="n">
-        <v>36822.63425331856</v>
+        <v>1453.525036315201</v>
       </c>
       <c r="D199" s="13" t="n">
-        <v>33876.82351305307</v>
+        <v>0</v>
       </c>
       <c r="E199" s="13" t="n">
-        <v>26423.9223401814</v>
+        <v>0</v>
       </c>
       <c r="F199" s="13" t="n">
-        <v>2945.810740265486</v>
-      </c>
-      <c r="G199" s="14" t="n">
-        <v>92</v>
-      </c>
-      <c r="H199" s="14" t="n">
-        <v>78</v>
-      </c>
-      <c r="I199" s="13" t="n">
-        <v>395.0574928079608</v>
-      </c>
+        <v>1453.525036315201</v>
+      </c>
+      <c r="G199" s="12" t="inlineStr"/>
+      <c r="H199" s="12" t="inlineStr"/>
+      <c r="I199" s="12" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="8" t="inlineStr">
         <is>
-          <t>C Magma to Remelt</t>
+          <t>C Magma</t>
         </is>
       </c>
       <c r="B200" s="8" t="inlineStr">
@@ -4140,16 +4045,16 @@
         </is>
       </c>
       <c r="C200" s="9" t="n">
-        <v>9205.65856332964</v>
+        <v>46028.29281664819</v>
       </c>
       <c r="D200" s="9" t="n">
-        <v>8469.205878263268</v>
+        <v>42346.02939131634</v>
       </c>
       <c r="E200" s="9" t="n">
-        <v>6605.98058504535</v>
+        <v>33029.90292522674</v>
       </c>
       <c r="F200" s="9" t="n">
-        <v>736.4526850663715</v>
+        <v>3682.263425331854</v>
       </c>
       <c r="G200" s="10" t="n">
         <v>92</v>
@@ -4158,7 +4063,7 @@
         <v>78</v>
       </c>
       <c r="I200" s="9" t="n">
-        <v>98.76437320199021</v>
+        <v>493.821866009951</v>
       </c>
     </row>
     <row r="201">
@@ -4192,16 +4097,16 @@
       </c>
       <c r="B202" s="17" t="inlineStr"/>
       <c r="C202" s="16" t="n">
-        <v>46028.2928166482</v>
+        <v>46028.29281664819</v>
       </c>
       <c r="D202" s="16" t="n">
         <v>42346.02939131634</v>
       </c>
       <c r="E202" s="16" t="n">
-        <v>33029.90292522675</v>
+        <v>33029.90292522674</v>
       </c>
       <c r="F202" s="16" t="n">
-        <v>3682.263425331861</v>
+        <v>3682.263425331854</v>
       </c>
       <c r="G202" s="17" t="inlineStr"/>
       <c r="H202" s="17" t="inlineStr"/>
@@ -4215,16 +4120,16 @@
       </c>
       <c r="B203" s="17" t="inlineStr"/>
       <c r="C203" s="16" t="n">
-        <v>-7.275957614183426e-12</v>
+        <v>0</v>
       </c>
       <c r="D203" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E203" s="16" t="n">
-        <v>-7.275957614183426e-12</v>
+        <v>0</v>
       </c>
       <c r="F203" s="16" t="n">
-        <v>-7.275957614183426e-12</v>
+        <v>0</v>
       </c>
       <c r="G203" s="17" t="inlineStr"/>
       <c r="H203" s="17" t="inlineStr"/>
@@ -4233,7 +4138,7 @@
     <row r="205" ht="17" customHeight="1">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>C REMELT  (target 65.0 Bx)</t>
+          <t>C MAGMA DISTRIBUTION</t>
         </is>
       </c>
       <c r="B205" s="5" t="n"/>
@@ -4295,7 +4200,7 @@
     <row r="207">
       <c r="A207" s="8" t="inlineStr">
         <is>
-          <t>C Magma (to Remelt)</t>
+          <t>Magma (total)</t>
         </is>
       </c>
       <c r="B207" s="8" t="inlineStr">
@@ -4304,16 +4209,16 @@
         </is>
       </c>
       <c r="C207" s="9" t="n">
-        <v>9205.65856332964</v>
+        <v>46028.29281664819</v>
       </c>
       <c r="D207" s="9" t="n">
-        <v>8469.205878263268</v>
+        <v>42346.02939131634</v>
       </c>
       <c r="E207" s="9" t="n">
-        <v>6605.98058504535</v>
+        <v>33029.90292522674</v>
       </c>
       <c r="F207" s="9" t="n">
-        <v>736.4526850663715</v>
+        <v>3682.263425331854</v>
       </c>
       <c r="G207" s="10" t="n">
         <v>92</v>
@@ -4322,40 +4227,46 @@
         <v>78</v>
       </c>
       <c r="I207" s="9" t="n">
-        <v>98.76437320199021</v>
+        <v>493.821866009951</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="12" t="inlineStr">
         <is>
-          <t>Remelt Water</t>
+          <t>C Magma to A Footing</t>
         </is>
       </c>
       <c r="B208" s="12" t="inlineStr">
         <is>
-          <t>In</t>
+          <t>Out</t>
         </is>
       </c>
       <c r="C208" s="13" t="n">
-        <v>3823.888941690773</v>
+        <v>36822.63425331856</v>
       </c>
       <c r="D208" s="13" t="n">
-        <v>0</v>
+        <v>33876.82351305307</v>
       </c>
       <c r="E208" s="13" t="n">
-        <v>0</v>
+        <v>26423.9223401814</v>
       </c>
       <c r="F208" s="13" t="n">
-        <v>3823.888941690773</v>
-      </c>
-      <c r="G208" s="12" t="inlineStr"/>
-      <c r="H208" s="12" t="inlineStr"/>
-      <c r="I208" s="12" t="inlineStr"/>
+        <v>2945.810740265486</v>
+      </c>
+      <c r="G208" s="14" t="n">
+        <v>92</v>
+      </c>
+      <c r="H208" s="14" t="n">
+        <v>78</v>
+      </c>
+      <c r="I208" s="13" t="n">
+        <v>395.0574928079608</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="8" t="inlineStr">
         <is>
-          <t>C Remelt</t>
+          <t>C Magma to Remelt</t>
         </is>
       </c>
       <c r="B209" s="8" t="inlineStr">
@@ -4364,7 +4275,7 @@
         </is>
       </c>
       <c r="C209" s="9" t="n">
-        <v>13029.54750502041</v>
+        <v>9205.65856332964</v>
       </c>
       <c r="D209" s="9" t="n">
         <v>8469.205878263268</v>
@@ -4373,16 +4284,16 @@
         <v>6605.98058504535</v>
       </c>
       <c r="F209" s="9" t="n">
-        <v>4560.341626757145</v>
+        <v>736.4526850663715</v>
       </c>
       <c r="G209" s="10" t="n">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="H209" s="10" t="n">
         <v>78</v>
       </c>
       <c r="I209" s="9" t="n">
-        <v>158.6821579326576</v>
+        <v>98.76437320199021</v>
       </c>
     </row>
     <row r="210">
@@ -4393,16 +4304,16 @@
       </c>
       <c r="B210" s="17" t="inlineStr"/>
       <c r="C210" s="16" t="n">
-        <v>13029.54750502041</v>
+        <v>46028.29281664819</v>
       </c>
       <c r="D210" s="16" t="n">
-        <v>8469.205878263268</v>
+        <v>42346.02939131634</v>
       </c>
       <c r="E210" s="16" t="n">
-        <v>6605.98058504535</v>
+        <v>33029.90292522674</v>
       </c>
       <c r="F210" s="16" t="n">
-        <v>4560.341626757145</v>
+        <v>3682.263425331854</v>
       </c>
       <c r="G210" s="17" t="inlineStr"/>
       <c r="H210" s="17" t="inlineStr"/>
@@ -4416,16 +4327,16 @@
       </c>
       <c r="B211" s="17" t="inlineStr"/>
       <c r="C211" s="16" t="n">
-        <v>13029.54750502041</v>
+        <v>46028.2928166482</v>
       </c>
       <c r="D211" s="16" t="n">
-        <v>8469.205878263268</v>
+        <v>42346.02939131634</v>
       </c>
       <c r="E211" s="16" t="n">
-        <v>6605.98058504535</v>
+        <v>33029.90292522675</v>
       </c>
       <c r="F211" s="16" t="n">
-        <v>4560.341626757145</v>
+        <v>3682.263425331861</v>
       </c>
       <c r="G211" s="17" t="inlineStr"/>
       <c r="H211" s="17" t="inlineStr"/>
@@ -4439,243 +4350,264 @@
       </c>
       <c r="B212" s="17" t="inlineStr"/>
       <c r="C212" s="16" t="n">
-        <v>0</v>
+        <v>-7.275957614183426e-12</v>
       </c>
       <c r="D212" s="16" t="n">
         <v>0</v>
       </c>
       <c r="E212" s="16" t="n">
-        <v>0</v>
+        <v>-7.275957614183426e-12</v>
       </c>
       <c r="F212" s="16" t="n">
-        <v>0</v>
+        <v>-7.275957614183426e-12</v>
       </c>
       <c r="G212" s="17" t="inlineStr"/>
       <c r="H212" s="17" t="inlineStr"/>
       <c r="I212" s="17" t="inlineStr"/>
     </row>
-    <row r="213">
-      <c r="A213" s="18" t="inlineStr">
-        <is>
-          <t>Target remelt brix</t>
-        </is>
-      </c>
-      <c r="B213" s="23" t="n">
+    <row r="214" ht="17" customHeight="1">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>C REMELT  (target 65.0 Bx)</t>
+        </is>
+      </c>
+      <c r="B214" s="5" t="n"/>
+      <c r="C214" s="5" t="n"/>
+      <c r="D214" s="5" t="n"/>
+      <c r="E214" s="5" t="n"/>
+      <c r="F214" s="5" t="n"/>
+      <c r="G214" s="5" t="n"/>
+      <c r="H214" s="5" t="n"/>
+      <c r="I214" s="5" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="6" t="inlineStr">
+        <is>
+          <t>Stream</t>
+        </is>
+      </c>
+      <c r="B215" s="6" t="inlineStr">
+        <is>
+          <t>Dir</t>
+        </is>
+      </c>
+      <c r="C215" s="6" t="inlineStr">
+        <is>
+          <t>Flow (lb/hr)</t>
+        </is>
+      </c>
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t>Solids (lb/hr)</t>
+        </is>
+      </c>
+      <c r="E215" s="6" t="inlineStr">
+        <is>
+          <t>Pol (lb/hr)</t>
+        </is>
+      </c>
+      <c r="F215" s="6" t="inlineStr">
+        <is>
+          <t>Water (lb/hr)</t>
+        </is>
+      </c>
+      <c r="G215" s="6" t="inlineStr">
+        <is>
+          <t>Brix %</t>
+        </is>
+      </c>
+      <c r="H215" s="6" t="inlineStr">
+        <is>
+          <t>Purity %</t>
+        </is>
+      </c>
+      <c r="I215" s="6" t="inlineStr">
+        <is>
+          <t>ft³/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="8" t="inlineStr">
+        <is>
+          <t>C Magma (to Remelt)</t>
+        </is>
+      </c>
+      <c r="B216" s="8" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="C216" s="9" t="n">
+        <v>9205.65856332964</v>
+      </c>
+      <c r="D216" s="9" t="n">
+        <v>8469.205878263268</v>
+      </c>
+      <c r="E216" s="9" t="n">
+        <v>6605.98058504535</v>
+      </c>
+      <c r="F216" s="9" t="n">
+        <v>736.4526850663715</v>
+      </c>
+      <c r="G216" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="H216" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="I216" s="9" t="n">
+        <v>98.76437320199021</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="12" t="inlineStr">
+        <is>
+          <t>Remelt Water</t>
+        </is>
+      </c>
+      <c r="B217" s="12" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="C217" s="13" t="n">
+        <v>3823.888941690773</v>
+      </c>
+      <c r="D217" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E217" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F217" s="13" t="n">
+        <v>3823.888941690773</v>
+      </c>
+      <c r="G217" s="12" t="inlineStr"/>
+      <c r="H217" s="12" t="inlineStr"/>
+      <c r="I217" s="12" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="8" t="inlineStr">
+        <is>
+          <t>C Remelt</t>
+        </is>
+      </c>
+      <c r="B218" s="8" t="inlineStr">
+        <is>
+          <t>Out</t>
+        </is>
+      </c>
+      <c r="C218" s="9" t="n">
+        <v>13029.54750502041</v>
+      </c>
+      <c r="D218" s="9" t="n">
+        <v>8469.205878263268</v>
+      </c>
+      <c r="E218" s="9" t="n">
+        <v>6605.98058504535</v>
+      </c>
+      <c r="F218" s="9" t="n">
+        <v>4560.341626757145</v>
+      </c>
+      <c r="G218" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="C213" s="20" t="inlineStr">
-        <is>
-          <t>Bx</t>
-        </is>
-      </c>
-    </row>
-    <row r="215" ht="17" customHeight="1">
-      <c r="A215" s="4" t="inlineStr">
-        <is>
-          <t>PAN VAPOR CONDENSERS  (one per pan)</t>
-        </is>
-      </c>
-      <c r="B215" s="5" t="n"/>
-      <c r="C215" s="5" t="n"/>
-      <c r="D215" s="5" t="n"/>
-      <c r="E215" s="5" t="n"/>
-      <c r="F215" s="5" t="n"/>
-      <c r="G215" s="5" t="n"/>
-      <c r="H215" s="5" t="n"/>
-      <c r="I215" s="5" t="n"/>
-    </row>
-    <row r="216">
-      <c r="A216" s="6" t="inlineStr">
-        <is>
-          <t>Condenser</t>
-        </is>
-      </c>
-      <c r="B216" s="6" t="inlineStr">
-        <is>
-          <t>Vapor (lb/hr)</t>
-        </is>
-      </c>
-      <c r="C216" s="6" t="inlineStr">
-        <is>
-          <t>Sat T (°F)</t>
-        </is>
-      </c>
-      <c r="D216" s="6" t="inlineStr">
-        <is>
-          <t>h_fg (BTU/lb)</t>
-        </is>
-      </c>
-      <c r="E216" s="6" t="inlineStr">
-        <is>
-          <t>Heat (MM BTU/hr)</t>
-        </is>
-      </c>
-      <c r="F216" s="6" t="inlineStr">
-        <is>
-          <t>Inj Water (lb/hr)</t>
-        </is>
-      </c>
-      <c r="G216" s="6" t="inlineStr">
-        <is>
-          <t>Inj Water (GPM)</t>
-        </is>
-      </c>
-      <c r="H216" s="6" t="inlineStr">
-        <is>
-          <t>Water Out (°F)</t>
-        </is>
-      </c>
-      <c r="I216" s="6" t="inlineStr">
-        <is>
-          <t>Total Out (lb/hr)</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="8" t="inlineStr">
-        <is>
-          <t>A Pans</t>
-        </is>
-      </c>
-      <c r="B217" s="9" t="n">
-        <v>68124.52640890723</v>
-      </c>
-      <c r="C217" s="10" t="n">
-        <v>143.355890609762</v>
-      </c>
-      <c r="D217" s="10" t="n">
-        <v>1011.249247318053</v>
-      </c>
-      <c r="E217" s="24" t="n">
-        <v>69.23149868695079</v>
-      </c>
-      <c r="F217" s="9" t="n">
-        <v>1431707.653689135</v>
-      </c>
-      <c r="G217" s="9" t="n">
-        <v>2861.126406253268</v>
-      </c>
-      <c r="H217" s="10" t="n">
-        <v>138.355890609762</v>
-      </c>
-      <c r="I217" s="9" t="n">
-        <v>1499832.180098043</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" s="12" t="inlineStr">
-        <is>
-          <t>Grain Pans</t>
-        </is>
-      </c>
-      <c r="B218" s="13" t="n">
-        <v>1422.938650984632</v>
-      </c>
-      <c r="C218" s="14" t="n">
-        <v>129.059477265374</v>
-      </c>
-      <c r="D218" s="14" t="n">
-        <v>1019.563890979194</v>
-      </c>
-      <c r="E218" s="25" t="n">
-        <v>1.4578915608775</v>
-      </c>
-      <c r="F218" s="13" t="n">
-        <v>42804.28467877984</v>
-      </c>
-      <c r="G218" s="13" t="n">
-        <v>85.54013724776148</v>
-      </c>
-      <c r="H218" s="14" t="n">
-        <v>124.059477265374</v>
-      </c>
-      <c r="I218" s="13" t="n">
-        <v>44227.22332976447</v>
+      <c r="H218" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="I218" s="9" t="n">
+        <v>158.6821579326576</v>
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="8" t="inlineStr">
-        <is>
-          <t>C Pans</t>
-        </is>
-      </c>
-      <c r="B219" s="9" t="n">
-        <v>28696.07651165161</v>
-      </c>
-      <c r="C219" s="10" t="n">
-        <v>119.6832047961655</v>
-      </c>
-      <c r="D219" s="10" t="n">
-        <v>1024.996584701115</v>
-      </c>
-      <c r="E219" s="24" t="n">
-        <v>29.55686080132305</v>
-      </c>
-      <c r="F219" s="9" t="n">
-        <v>1197448.266762941</v>
-      </c>
-      <c r="G219" s="9" t="n">
-        <v>2392.982147807637</v>
-      </c>
-      <c r="H219" s="10" t="n">
-        <v>114.6832047961655</v>
-      </c>
-      <c r="I219" s="9" t="n">
-        <v>1226144.343274593</v>
-      </c>
+      <c r="A219" s="17" t="inlineStr">
+        <is>
+          <t>Total In</t>
+        </is>
+      </c>
+      <c r="B219" s="17" t="inlineStr"/>
+      <c r="C219" s="16" t="n">
+        <v>13029.54750502041</v>
+      </c>
+      <c r="D219" s="16" t="n">
+        <v>8469.205878263268</v>
+      </c>
+      <c r="E219" s="16" t="n">
+        <v>6605.98058504535</v>
+      </c>
+      <c r="F219" s="16" t="n">
+        <v>4560.341626757145</v>
+      </c>
+      <c r="G219" s="17" t="inlineStr"/>
+      <c r="H219" s="17" t="inlineStr"/>
+      <c r="I219" s="17" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="17" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B220" s="16" t="n">
-        <v>98243.54157154348</v>
-      </c>
-      <c r="C220" s="17" t="inlineStr"/>
-      <c r="D220" s="17" t="inlineStr"/>
-      <c r="E220" s="26" t="n">
-        <v>100.2462510491513</v>
+          <t>Total Out</t>
+        </is>
+      </c>
+      <c r="B220" s="17" t="inlineStr"/>
+      <c r="C220" s="16" t="n">
+        <v>13029.54750502041</v>
+      </c>
+      <c r="D220" s="16" t="n">
+        <v>8469.205878263268</v>
+      </c>
+      <c r="E220" s="16" t="n">
+        <v>6605.98058504535</v>
       </c>
       <c r="F220" s="16" t="n">
-        <v>2671960.205130856</v>
-      </c>
-      <c r="G220" s="16" t="n">
-        <v>5339.648691308666</v>
-      </c>
+        <v>4560.341626757145</v>
+      </c>
+      <c r="G220" s="17" t="inlineStr"/>
       <c r="H220" s="17" t="inlineStr"/>
-      <c r="I220" s="16" t="n">
-        <v>2770203.7467024</v>
-      </c>
+      <c r="I220" s="17" t="inlineStr"/>
     </row>
     <row r="221">
-      <c r="A221" s="18" t="inlineStr">
-        <is>
-          <t>Injection water supply temp</t>
-        </is>
-      </c>
-      <c r="B221" s="23" t="n">
-        <v>90</v>
-      </c>
-      <c r="C221" s="20" t="inlineStr">
-        <is>
-          <t>°F</t>
-        </is>
-      </c>
+      <c r="A221" s="17" t="inlineStr">
+        <is>
+          <t>Net (In - Out)</t>
+        </is>
+      </c>
+      <c r="B221" s="17" t="inlineStr"/>
+      <c r="C221" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D221" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E221" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F221" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G221" s="17" t="inlineStr"/>
+      <c r="H221" s="17" t="inlineStr"/>
+      <c r="I221" s="17" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="18" t="inlineStr">
         <is>
-          <t>Note: if using CoolingTowerSystem, ignore these injection water demands - they are re-solved there at the delivered water temp.</t>
-        </is>
-      </c>
-      <c r="B222" s="18" t="inlineStr"/>
+          <t>Target remelt brix</t>
+        </is>
+      </c>
+      <c r="B222" s="23" t="n">
+        <v>65</v>
+      </c>
+      <c r="C222" s="20" t="inlineStr">
+        <is>
+          <t>Bx</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="17" customHeight="1">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>CONDENSATE RETURN</t>
+          <t>PAN VAPOR CONDENSERS  (one per pan)</t>
         </is>
       </c>
       <c r="B224" s="5" t="n"/>
@@ -4688,45 +4620,248 @@
       <c r="I224" s="5" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="18" t="inlineStr">
+      <c r="A225" s="6" t="inlineStr">
+        <is>
+          <t>Condenser</t>
+        </is>
+      </c>
+      <c r="B225" s="6" t="inlineStr">
+        <is>
+          <t>Vapor (lb/hr)</t>
+        </is>
+      </c>
+      <c r="C225" s="6" t="inlineStr">
+        <is>
+          <t>Sat T (°F)</t>
+        </is>
+      </c>
+      <c r="D225" s="6" t="inlineStr">
+        <is>
+          <t>h_fg (BTU/lb)</t>
+        </is>
+      </c>
+      <c r="E225" s="6" t="inlineStr">
+        <is>
+          <t>Heat (MM BTU/hr)</t>
+        </is>
+      </c>
+      <c r="F225" s="6" t="inlineStr">
+        <is>
+          <t>Inj Water (lb/hr)</t>
+        </is>
+      </c>
+      <c r="G225" s="6" t="inlineStr">
+        <is>
+          <t>Inj Water (GPM)</t>
+        </is>
+      </c>
+      <c r="H225" s="6" t="inlineStr">
+        <is>
+          <t>Water Out (°F)</t>
+        </is>
+      </c>
+      <c r="I225" s="6" t="inlineStr">
+        <is>
+          <t>Total Out (lb/hr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="8" t="inlineStr">
+        <is>
+          <t>A Pans</t>
+        </is>
+      </c>
+      <c r="B226" s="9" t="n">
+        <v>68124.52640890723</v>
+      </c>
+      <c r="C226" s="10" t="n">
+        <v>143.355890609762</v>
+      </c>
+      <c r="D226" s="10" t="n">
+        <v>1011.249247318053</v>
+      </c>
+      <c r="E226" s="24" t="n">
+        <v>69.23149868695079</v>
+      </c>
+      <c r="F226" s="9" t="n">
+        <v>1431707.653689135</v>
+      </c>
+      <c r="G226" s="9" t="n">
+        <v>2861.126406253268</v>
+      </c>
+      <c r="H226" s="10" t="n">
+        <v>138.355890609762</v>
+      </c>
+      <c r="I226" s="9" t="n">
+        <v>1499832.180098043</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="12" t="inlineStr">
+        <is>
+          <t>Grain Pans</t>
+        </is>
+      </c>
+      <c r="B227" s="13" t="n">
+        <v>1422.938650984632</v>
+      </c>
+      <c r="C227" s="14" t="n">
+        <v>129.059477265374</v>
+      </c>
+      <c r="D227" s="14" t="n">
+        <v>1019.563890979194</v>
+      </c>
+      <c r="E227" s="25" t="n">
+        <v>1.4578915608775</v>
+      </c>
+      <c r="F227" s="13" t="n">
+        <v>42804.28467877984</v>
+      </c>
+      <c r="G227" s="13" t="n">
+        <v>85.54013724776148</v>
+      </c>
+      <c r="H227" s="14" t="n">
+        <v>124.059477265374</v>
+      </c>
+      <c r="I227" s="13" t="n">
+        <v>44227.22332976447</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="8" t="inlineStr">
+        <is>
+          <t>C Pans</t>
+        </is>
+      </c>
+      <c r="B228" s="9" t="n">
+        <v>28696.07651165161</v>
+      </c>
+      <c r="C228" s="10" t="n">
+        <v>119.6832047961655</v>
+      </c>
+      <c r="D228" s="10" t="n">
+        <v>1024.996584701115</v>
+      </c>
+      <c r="E228" s="24" t="n">
+        <v>29.55686080132305</v>
+      </c>
+      <c r="F228" s="9" t="n">
+        <v>1197448.266762941</v>
+      </c>
+      <c r="G228" s="9" t="n">
+        <v>2392.982147807637</v>
+      </c>
+      <c r="H228" s="10" t="n">
+        <v>114.6832047961655</v>
+      </c>
+      <c r="I228" s="9" t="n">
+        <v>1226144.343274593</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="17" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B229" s="16" t="n">
+        <v>98243.54157154348</v>
+      </c>
+      <c r="C229" s="17" t="inlineStr"/>
+      <c r="D229" s="17" t="inlineStr"/>
+      <c r="E229" s="26" t="n">
+        <v>100.2462510491513</v>
+      </c>
+      <c r="F229" s="16" t="n">
+        <v>2671960.205130856</v>
+      </c>
+      <c r="G229" s="16" t="n">
+        <v>5339.648691308666</v>
+      </c>
+      <c r="H229" s="17" t="inlineStr"/>
+      <c r="I229" s="16" t="n">
+        <v>2770203.7467024</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="18" t="inlineStr">
+        <is>
+          <t>Injection water supply temp</t>
+        </is>
+      </c>
+      <c r="B230" s="23" t="n">
+        <v>90</v>
+      </c>
+      <c r="C230" s="20" t="inlineStr">
+        <is>
+          <t>°F</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="18" t="inlineStr">
+        <is>
+          <t>Note: if using CoolingTowerSystem, ignore these injection water demands - they are re-solved there at the delivered water temp.</t>
+        </is>
+      </c>
+      <c r="B231" s="18" t="inlineStr"/>
+    </row>
+    <row r="233" ht="17" customHeight="1">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>CONDENSATE RETURN</t>
+        </is>
+      </c>
+      <c r="B233" s="5" t="n"/>
+      <c r="C233" s="5" t="n"/>
+      <c r="D233" s="5" t="n"/>
+      <c r="E233" s="5" t="n"/>
+      <c r="F233" s="5" t="n"/>
+      <c r="G233" s="5" t="n"/>
+      <c r="H233" s="5" t="n"/>
+      <c r="I233" s="5" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="18" t="inlineStr">
         <is>
           <t>Clean condensate (Exhaust steam pans)</t>
         </is>
       </c>
-      <c r="B225" s="22" t="n">
+      <c r="B234" s="22" t="n">
         <v>111502.0701128084</v>
       </c>
-      <c r="C225" s="20" t="inlineStr">
+      <c r="C234" s="20" t="inlineStr">
         <is>
           <t>lb/hr</t>
         </is>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="18" t="inlineStr">
+    <row r="235">
+      <c r="A235" s="18" t="inlineStr">
         <is>
           <t>Dirty condensate (V1-V4 steam pans)</t>
         </is>
       </c>
-      <c r="B226" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C226" s="20" t="inlineStr">
+      <c r="B235" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C235" s="20" t="inlineStr">
         <is>
           <t>lb/hr</t>
         </is>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="18" t="inlineStr">
+    <row r="236">
+      <c r="A236" s="18" t="inlineStr">
         <is>
           <t>Total condensate</t>
         </is>
       </c>
-      <c r="B227" s="22" t="n">
+      <c r="B236" s="22" t="n">
         <v>111502.0701128084</v>
       </c>
-      <c r="C227" s="20" t="inlineStr">
+      <c r="C236" s="20" t="inlineStr">
         <is>
           <t>lb/hr</t>
         </is>
@@ -4739,20 +4874,20 @@
     <mergeCell ref="A90:I90"/>
     <mergeCell ref="A99:I99"/>
     <mergeCell ref="A177:I177"/>
-    <mergeCell ref="A145:I145"/>
-    <mergeCell ref="A113:I113"/>
+    <mergeCell ref="A233:I233"/>
+    <mergeCell ref="A214:I214"/>
+    <mergeCell ref="A151:I151"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A159:I159"/>
-    <mergeCell ref="A215:I215"/>
+    <mergeCell ref="A116:I116"/>
+    <mergeCell ref="A126:I126"/>
+    <mergeCell ref="A135:I135"/>
     <mergeCell ref="A224:I224"/>
     <mergeCell ref="A44:I44"/>
-    <mergeCell ref="A123:I123"/>
+    <mergeCell ref="A186:I186"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A132:I132"/>
     <mergeCell ref="A168:I168"/>
     <mergeCell ref="A78:I78"/>
-    <mergeCell ref="A187:I187"/>
     <mergeCell ref="A205:I205"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
@@ -4761,7 +4896,7 @@
     <brk id="42" min="0" max="16383" man="1"/>
     <brk id="63" min="0" max="16383" man="1"/>
     <brk id="97" min="0" max="16383" man="1"/>
-    <brk id="130" min="0" max="16383" man="1"/>
+    <brk id="133" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>